<commit_message>
test(02-05): add failing tests for file_parser and frequency_resolver
- test_file_parser: CSV/Excel/JSON type detection, malformed CSV auto-fix
- test_frequency_resolver: daily vs quarterly conflict detection, mean/ffill resolution
- Add fixture files: sample.csv, malformed.csv, sample.json, sample.xlsx
- Add schemas/data.py with FrequencyConflict, UploadResult, AssumptionItem
- Add pandas, openpyxl, fredapi, anthropic to pyproject.toml
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/sample.xlsx
+++ b/backend/tests/fixtures/sample.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,133 +563,6 @@
         <v>260.4</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2020-11-01</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>21731.2</v>
-      </c>
-      <c r="C12" t="n">
-        <v>260.2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2020-12-01</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>21854.1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2021-01-01</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>21921</v>
-      </c>
-      <c r="C14" t="n">
-        <v>261.6</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2021-02-01</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>22046.5</v>
-      </c>
-      <c r="C15" t="n">
-        <v>263.1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2021-03-01</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>22369.2</v>
-      </c>
-      <c r="C16" t="n">
-        <v>264.9</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2021-04-01</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>22741</v>
-      </c>
-      <c r="C17" t="n">
-        <v>267.1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2021-05-01</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>22997.5</v>
-      </c>
-      <c r="C18" t="n">
-        <v>268.6</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2021-06-01</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>23185.1</v>
-      </c>
-      <c r="C19" t="n">
-        <v>271.7</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2021-07-01</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>23349.7</v>
-      </c>
-      <c r="C20" t="n">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2021-08-01</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>23492.2</v>
-      </c>
-      <c r="C21" t="n">
-        <v>273.6</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>